<commit_message>
added code fil e need to update
</commit_message>
<xml_diff>
--- a/1234567 (1).xlsx
+++ b/1234567 (1).xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="63">
   <si>
     <t xml:space="preserve">My Data, My Code</t>
   </si>
@@ -119,7 +119,7 @@
     <t xml:space="preserve">Name:</t>
   </si>
   <si>
-    <t xml:space="preserve">Shameem ali</t>
+    <t xml:space="preserve">Shameem Ali T</t>
   </si>
   <si>
     <t xml:space="preserve">Registration No.:</t>
@@ -188,10 +188,28 @@
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">Example row — replace with your own data. Felt a bit tired after evening class.</t>
+    <t xml:space="preserve">Felt a bit tired after evening class.</t>
   </si>
   <si>
     <t xml:space="preserve">Neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsatisfied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excellent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very Satisfied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very Unsatisfied</t>
   </si>
 </sst>
 </file>
@@ -203,7 +221,7 @@
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,13 +314,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <i val="true"/>
       <sz val="11"/>
       <color rgb="FF808080"/>
@@ -316,6 +327,7 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -457,35 +469,35 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1194,39 +1206,43 @@
         <v>46225</v>
       </c>
       <c r="B8" s="9" t="n">
-        <v>501</v>
+        <v>495</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I8" s="21" t="n">
         <f aca="false">IF(SUM(B8:F8,H8)=0,"",SUM(B8:F8,H8))</f>
-        <v>901</v>
+        <v>875</v>
       </c>
       <c r="J8" s="21" t="n">
         <f aca="false">IF(I8="","",1440-I8)</f>
-        <v>539</v>
+        <v>565</v>
       </c>
       <c r="K8" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22"/>
+        <v>56</v>
+      </c>
+      <c r="L8" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M8" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N8" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1234,39 +1250,43 @@
         <v>46226</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>502</v>
+        <v>470</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>25</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>152</v>
+        <v>100</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I9" s="21" t="n">
         <f aca="false">IF(SUM(B9:F9,H9)=0,"",SUM(B9:F9,H9))</f>
-        <v>900</v>
+        <v>795</v>
       </c>
       <c r="J9" s="21" t="n">
         <f aca="false">IF(I9="","",1440-I9)</f>
-        <v>540</v>
+        <v>645</v>
       </c>
       <c r="K9" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
+        <v>56</v>
+      </c>
+      <c r="L9" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M9" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N9" s="23"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1274,39 +1294,43 @@
         <v>46227</v>
       </c>
       <c r="B10" s="9" t="n">
-        <v>503</v>
+        <v>490</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>153</v>
+        <v>120</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I10" s="21" t="n">
         <f aca="false">IF(SUM(B10:F10,H10)=0,"",SUM(B10:F10,H10))</f>
-        <v>906</v>
+        <v>830</v>
       </c>
       <c r="J10" s="21" t="n">
         <f aca="false">IF(I10="","",1440-I10)</f>
-        <v>534</v>
+        <v>610</v>
       </c>
       <c r="K10" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
+      <c r="L10" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M10" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1314,39 +1338,43 @@
         <v>46228</v>
       </c>
       <c r="B11" s="9" t="n">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="I11" s="21" t="n">
         <f aca="false">IF(SUM(B11:F11,H11)=0,"",SUM(B11:F11,H11))</f>
-        <v>919</v>
+        <v>907</v>
       </c>
       <c r="J11" s="21" t="n">
         <f aca="false">IF(I11="","",1440-I11)</f>
-        <v>521</v>
+        <v>533</v>
       </c>
       <c r="K11" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22"/>
+      <c r="L11" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M11" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N11" s="23"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1369,7 +1397,7 @@
         <v>155</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>30</v>
@@ -1383,10 +1411,14 @@
         <v>515</v>
       </c>
       <c r="K12" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="L12" s="22"/>
-      <c r="M12" s="22"/>
+        <v>56</v>
+      </c>
+      <c r="L12" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M12" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1394,39 +1426,43 @@
         <v>46230</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>506</v>
+        <v>550</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>156</v>
+        <v>200</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="I13" s="21" t="n">
         <f aca="false">IF(SUM(B13:F13,H13)=0,"",SUM(B13:F13,H13))</f>
-        <v>931</v>
+        <v>990</v>
       </c>
       <c r="J13" s="21" t="n">
         <f aca="false">IF(I13="","",1440-I13)</f>
-        <v>509</v>
+        <v>450</v>
       </c>
       <c r="K13" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L13" s="22"/>
-      <c r="M13" s="22"/>
+      <c r="L13" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M13" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1434,39 +1470,43 @@
         <v>46231</v>
       </c>
       <c r="B14" s="9" t="n">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="I14" s="21" t="n">
         <f aca="false">IF(SUM(B14:F14,H14)=0,"",SUM(B14:F14,H14))</f>
-        <v>937</v>
+        <v>920</v>
       </c>
       <c r="J14" s="21" t="n">
         <f aca="false">IF(I14="","",1440-I14)</f>
-        <v>503</v>
+        <v>520</v>
       </c>
       <c r="K14" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L14" s="22"/>
-      <c r="M14" s="22"/>
+      <c r="L14" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M14" s="22" t="s">
+        <v>57</v>
+      </c>
       <c r="N14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1474,39 +1514,43 @@
         <v>46232</v>
       </c>
       <c r="B15" s="9" t="n">
-        <v>508</v>
+        <v>450</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H15" s="9" t="n">
         <v>33</v>
       </c>
       <c r="I15" s="21" t="n">
         <f aca="false">IF(SUM(B15:F15,H15)=0,"",SUM(B15:F15,H15))</f>
-        <v>943</v>
+        <v>825</v>
       </c>
       <c r="J15" s="21" t="n">
         <f aca="false">IF(I15="","",1440-I15)</f>
-        <v>497</v>
+        <v>615</v>
       </c>
       <c r="K15" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="L15" s="22"/>
-      <c r="M15" s="22"/>
+        <v>58</v>
+      </c>
+      <c r="L15" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="M15" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1514,39 +1558,43 @@
         <v>46233</v>
       </c>
       <c r="B16" s="9" t="n">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I16" s="21" t="n">
         <f aca="false">IF(SUM(B16:F16,H16)=0,"",SUM(B16:F16,H16))</f>
-        <v>949</v>
+        <v>915</v>
       </c>
       <c r="J16" s="21" t="n">
         <f aca="false">IF(I16="","",1440-I16)</f>
-        <v>491</v>
+        <v>525</v>
       </c>
       <c r="K16" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22"/>
+      <c r="L16" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M16" s="22" t="s">
+        <v>57</v>
+      </c>
       <c r="N16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1569,7 +1617,7 @@
         <v>160</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H17" s="9" t="n">
         <v>35</v>
@@ -1583,10 +1631,14 @@
         <v>485</v>
       </c>
       <c r="K17" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22"/>
+        <v>60</v>
+      </c>
+      <c r="L17" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M17" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N17" s="23"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1594,39 +1646,43 @@
         <v>46235</v>
       </c>
       <c r="B18" s="9" t="n">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>161</v>
+        <v>140</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="I18" s="21" t="n">
         <f aca="false">IF(SUM(B18:F18,H18)=0,"",SUM(B18:F18,H18))</f>
-        <v>961</v>
+        <v>925</v>
       </c>
       <c r="J18" s="21" t="n">
         <f aca="false">IF(I18="","",1440-I18)</f>
-        <v>479</v>
+        <v>515</v>
       </c>
       <c r="K18" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
+      <c r="L18" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M18" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N18" s="23"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1637,36 +1693,40 @@
         <v>512</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>162</v>
+        <v>100</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="I19" s="21" t="n">
         <f aca="false">IF(SUM(B19:F19,H19)=0,"",SUM(B19:F19,H19))</f>
-        <v>967</v>
+        <v>812</v>
       </c>
       <c r="J19" s="21" t="n">
         <f aca="false">IF(I19="","",1440-I19)</f>
-        <v>473</v>
+        <v>628</v>
       </c>
       <c r="K19" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
+      <c r="L19" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M19" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N19" s="23"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1674,39 +1734,43 @@
         <v>46237</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>513</v>
+        <v>400</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="D20" s="9" t="n">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>163</v>
+        <v>60</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="I20" s="21" t="n">
         <f aca="false">IF(SUM(B20:F20,H20)=0,"",SUM(B20:F20,H20))</f>
-        <v>973</v>
+        <v>770</v>
       </c>
       <c r="J20" s="21" t="n">
         <f aca="false">IF(I20="","",1440-I20)</f>
-        <v>467</v>
+        <v>670</v>
       </c>
       <c r="K20" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
+      <c r="L20" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M20" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1714,39 +1778,43 @@
         <v>46238</v>
       </c>
       <c r="B21" s="9" t="n">
-        <v>514</v>
+        <v>420</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>30</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>114</v>
+        <v>80</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>104</v>
+        <v>40</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I21" s="21" t="n">
         <f aca="false">IF(SUM(B21:F21,H21)=0,"",SUM(B21:F21,H21))</f>
-        <v>965</v>
+        <v>740</v>
       </c>
       <c r="J21" s="21" t="n">
         <f aca="false">IF(I21="","",1440-I21)</f>
-        <v>475</v>
+        <v>700</v>
       </c>
       <c r="K21" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
+      <c r="L21" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="M21" s="22" t="s">
+        <v>58</v>
+      </c>
       <c r="N21" s="23"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1757,36 +1825,40 @@
         <v>515</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>115</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="H22" s="9" t="n">
         <v>40</v>
       </c>
       <c r="I22" s="21" t="n">
         <f aca="false">IF(SUM(B22:F22,H22)=0,"",SUM(B22:F22,H22))</f>
-        <v>971</v>
+        <v>915</v>
       </c>
       <c r="J22" s="21" t="n">
         <f aca="false">IF(I22="","",1440-I22)</f>
-        <v>469</v>
+        <v>525</v>
       </c>
       <c r="K22" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
+      <c r="L22" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M22" s="22" t="s">
+        <v>58</v>
+      </c>
       <c r="N22" s="23"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1794,39 +1866,43 @@
         <v>46240</v>
       </c>
       <c r="B23" s="9" t="n">
-        <v>516</v>
+        <v>480</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>106</v>
+        <v>60</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="G23" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="9" t="n">
         <v>20</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>41</v>
       </c>
       <c r="I23" s="21" t="n">
         <f aca="false">IF(SUM(B23:F23,H23)=0,"",SUM(B23:F23,H23))</f>
-        <v>977</v>
+        <v>820</v>
       </c>
       <c r="J23" s="21" t="n">
         <f aca="false">IF(I23="","",1440-I23)</f>
-        <v>463</v>
+        <v>620</v>
       </c>
       <c r="K23" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
+      <c r="L23" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M23" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N23" s="23"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1834,39 +1910,43 @@
         <v>46241</v>
       </c>
       <c r="B24" s="9" t="n">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>107</v>
+        <v>75</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>167</v>
+        <v>70</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="I24" s="21" t="n">
         <f aca="false">IF(SUM(B24:F24,H24)=0,"",SUM(B24:F24,H24))</f>
-        <v>983</v>
+        <v>835</v>
       </c>
       <c r="J24" s="21" t="n">
         <f aca="false">IF(I24="","",1440-I24)</f>
-        <v>457</v>
+        <v>605</v>
       </c>
       <c r="K24" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
+      <c r="L24" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M24" s="22" t="s">
+        <v>57</v>
+      </c>
       <c r="N24" s="23"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1874,39 +1954,43 @@
         <v>46242</v>
       </c>
       <c r="B25" s="9" t="n">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>168</v>
+        <v>200</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="I25" s="21" t="n">
         <f aca="false">IF(SUM(B25:F25,H25)=0,"",SUM(B25:F25,H25))</f>
-        <v>989</v>
+        <v>940</v>
       </c>
       <c r="J25" s="21" t="n">
         <f aca="false">IF(I25="","",1440-I25)</f>
-        <v>451</v>
+        <v>500</v>
       </c>
       <c r="K25" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
+      <c r="L25" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="M25" s="22" t="s">
+        <v>58</v>
+      </c>
       <c r="N25" s="23"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1945,8 +2029,12 @@
       <c r="K26" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L26" s="22"/>
-      <c r="M26" s="22"/>
+      <c r="L26" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M26" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N26" s="23"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1954,7 +2042,7 @@
         <v>46244</v>
       </c>
       <c r="B27" s="9" t="n">
-        <v>520</v>
+        <v>500</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>36</v>
@@ -1976,17 +2064,21 @@
       </c>
       <c r="I27" s="21" t="n">
         <f aca="false">IF(SUM(B27:F27,H27)=0,"",SUM(B27:F27,H27))</f>
-        <v>1001</v>
+        <v>981</v>
       </c>
       <c r="J27" s="21" t="n">
         <f aca="false">IF(I27="","",1440-I27)</f>
-        <v>439</v>
+        <v>459</v>
       </c>
       <c r="K27" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
+      <c r="L27" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M27" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N27" s="23"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1994,7 +2086,7 @@
         <v>46245</v>
       </c>
       <c r="B28" s="9" t="n">
-        <v>521</v>
+        <v>501</v>
       </c>
       <c r="C28" s="9" t="n">
         <v>37</v>
@@ -2016,17 +2108,21 @@
       </c>
       <c r="I28" s="21" t="n">
         <f aca="false">IF(SUM(B28:F28,H28)=0,"",SUM(B28:F28,H28))</f>
-        <v>1007</v>
+        <v>987</v>
       </c>
       <c r="J28" s="21" t="n">
         <f aca="false">IF(I28="","",1440-I28)</f>
-        <v>433</v>
+        <v>453</v>
       </c>
       <c r="K28" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L28" s="22"/>
-      <c r="M28" s="22"/>
+      <c r="L28" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M28" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N28" s="23"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2034,7 +2130,7 @@
         <v>46246</v>
       </c>
       <c r="B29" s="9" t="n">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="C29" s="9" t="n">
         <v>38</v>
@@ -2056,17 +2152,21 @@
       </c>
       <c r="I29" s="21" t="n">
         <f aca="false">IF(SUM(B29:F29,H29)=0,"",SUM(B29:F29,H29))</f>
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="J29" s="21" t="n">
         <f aca="false">IF(I29="","",1440-I29)</f>
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="K29" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L29" s="22"/>
-      <c r="M29" s="22"/>
+      <c r="L29" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M29" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N29" s="23"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2074,7 +2174,7 @@
         <v>46247</v>
       </c>
       <c r="B30" s="9" t="n">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>39</v>
@@ -2096,17 +2196,21 @@
       </c>
       <c r="I30" s="21" t="n">
         <f aca="false">IF(SUM(B30:F30,H30)=0,"",SUM(B30:F30,H30))</f>
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="J30" s="21" t="n">
         <f aca="false">IF(I30="","",1440-I30)</f>
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="K30" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L30" s="22"/>
-      <c r="M30" s="22"/>
+      <c r="L30" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M30" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N30" s="23"/>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2114,7 +2218,7 @@
         <v>46248</v>
       </c>
       <c r="B31" s="9" t="n">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>54</v>
@@ -2136,17 +2240,21 @@
       </c>
       <c r="I31" s="21" t="n">
         <f aca="false">IF(SUM(B31:F31,H31)=0,"",SUM(B31:F31,H31))</f>
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="J31" s="21" t="n">
         <f aca="false">IF(I31="","",1440-I31)</f>
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="K31" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L31" s="22"/>
-      <c r="M31" s="22"/>
+      <c r="L31" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M31" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N31" s="23"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2154,7 +2262,7 @@
         <v>46249</v>
       </c>
       <c r="B32" s="9" t="n">
-        <v>525</v>
+        <v>545</v>
       </c>
       <c r="C32" s="9" t="n">
         <v>55</v>
@@ -2163,7 +2271,7 @@
         <v>125</v>
       </c>
       <c r="E32" s="9" t="n">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="F32" s="9" t="n">
         <v>175</v>
@@ -2176,17 +2284,21 @@
       </c>
       <c r="I32" s="21" t="n">
         <f aca="false">IF(SUM(B32:F32,H32)=0,"",SUM(B32:F32,H32))</f>
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="J32" s="21" t="n">
         <f aca="false">IF(I32="","",1440-I32)</f>
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="K32" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L32" s="22"/>
-      <c r="M32" s="22"/>
+      <c r="L32" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M32" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N32" s="23"/>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2194,7 +2306,7 @@
         <v>46250</v>
       </c>
       <c r="B33" s="9" t="n">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>56</v>
@@ -2203,7 +2315,7 @@
         <v>126</v>
       </c>
       <c r="E33" s="9" t="n">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>176</v>
@@ -2216,17 +2328,21 @@
       </c>
       <c r="I33" s="21" t="n">
         <f aca="false">IF(SUM(B33:F33,H33)=0,"",SUM(B33:F33,H33))</f>
-        <v>1051</v>
+        <v>1034</v>
       </c>
       <c r="J33" s="21" t="n">
         <f aca="false">IF(I33="","",1440-I33)</f>
-        <v>389</v>
+        <v>406</v>
       </c>
       <c r="K33" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L33" s="22"/>
-      <c r="M33" s="22"/>
+      <c r="L33" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M33" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N33" s="23"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2234,7 +2350,7 @@
         <v>46251</v>
       </c>
       <c r="B34" s="9" t="n">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C34" s="9" t="n">
         <v>57</v>
@@ -2243,7 +2359,7 @@
         <v>127</v>
       </c>
       <c r="E34" s="9" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="F34" s="9" t="n">
         <v>177</v>
@@ -2256,17 +2372,21 @@
       </c>
       <c r="I34" s="21" t="n">
         <f aca="false">IF(SUM(B34:F34,H34)=0,"",SUM(B34:F34,H34))</f>
-        <v>1057</v>
+        <v>1040</v>
       </c>
       <c r="J34" s="21" t="n">
         <f aca="false">IF(I34="","",1440-I34)</f>
-        <v>383</v>
+        <v>400</v>
       </c>
       <c r="K34" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L34" s="22"/>
-      <c r="M34" s="22"/>
+      <c r="L34" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M34" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N34" s="23"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2274,7 +2394,7 @@
         <v>46252</v>
       </c>
       <c r="B35" s="9" t="n">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>58</v>
@@ -2283,7 +2403,7 @@
         <v>128</v>
       </c>
       <c r="E35" s="9" t="n">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>178</v>
@@ -2296,17 +2416,21 @@
       </c>
       <c r="I35" s="21" t="n">
         <f aca="false">IF(SUM(B35:F35,H35)=0,"",SUM(B35:F35,H35))</f>
-        <v>1063</v>
+        <v>1046</v>
       </c>
       <c r="J35" s="21" t="n">
         <f aca="false">IF(I35="","",1440-I35)</f>
-        <v>377</v>
+        <v>394</v>
       </c>
       <c r="K35" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L35" s="22"/>
-      <c r="M35" s="22"/>
+      <c r="L35" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M35" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N35" s="23"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2314,16 +2438,16 @@
         <v>46253</v>
       </c>
       <c r="B36" s="9" t="n">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C36" s="9" t="n">
         <v>59</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="F36" s="9" t="n">
         <v>179</v>
@@ -2336,17 +2460,21 @@
       </c>
       <c r="I36" s="21" t="n">
         <f aca="false">IF(SUM(B36:F36,H36)=0,"",SUM(B36:F36,H36))</f>
-        <v>1069</v>
+        <v>1053</v>
       </c>
       <c r="J36" s="21" t="n">
         <f aca="false">IF(I36="","",1440-I36)</f>
-        <v>371</v>
+        <v>387</v>
       </c>
       <c r="K36" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L36" s="22"/>
-      <c r="M36" s="22"/>
+      <c r="L36" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M36" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N36" s="23"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2363,7 +2491,7 @@
         <v>130</v>
       </c>
       <c r="E37" s="9" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>180</v>
@@ -2376,17 +2504,21 @@
       </c>
       <c r="I37" s="21" t="n">
         <f aca="false">IF(SUM(B37:F37,H37)=0,"",SUM(B37:F37,H37))</f>
-        <v>1075</v>
+        <v>1025</v>
       </c>
       <c r="J37" s="21" t="n">
         <f aca="false">IF(I37="","",1440-I37)</f>
-        <v>365</v>
+        <v>415</v>
       </c>
       <c r="K37" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L37" s="22"/>
-      <c r="M37" s="22"/>
+      <c r="L37" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M37" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N37" s="23"/>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2403,7 +2535,7 @@
         <v>131</v>
       </c>
       <c r="E38" s="9" t="n">
-        <v>121</v>
+        <v>71</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>181</v>
@@ -2416,17 +2548,21 @@
       </c>
       <c r="I38" s="21" t="n">
         <f aca="false">IF(SUM(B38:F38,H38)=0,"",SUM(B38:F38,H38))</f>
-        <v>1081</v>
+        <v>1031</v>
       </c>
       <c r="J38" s="21" t="n">
         <f aca="false">IF(I38="","",1440-I38)</f>
-        <v>359</v>
+        <v>409</v>
       </c>
       <c r="K38" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L38" s="22"/>
-      <c r="M38" s="22"/>
+      <c r="L38" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M38" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N38" s="23"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2443,7 +2579,7 @@
         <v>132</v>
       </c>
       <c r="E39" s="9" t="n">
-        <v>122</v>
+        <v>72</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>182</v>
@@ -2456,17 +2592,21 @@
       </c>
       <c r="I39" s="21" t="n">
         <f aca="false">IF(SUM(B39:F39,H39)=0,"",SUM(B39:F39,H39))</f>
-        <v>1087</v>
+        <v>1037</v>
       </c>
       <c r="J39" s="21" t="n">
         <f aca="false">IF(I39="","",1440-I39)</f>
-        <v>353</v>
+        <v>403</v>
       </c>
       <c r="K39" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L39" s="22"/>
-      <c r="M39" s="22"/>
+      <c r="L39" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M39" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N39" s="23"/>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2483,7 +2623,7 @@
         <v>133</v>
       </c>
       <c r="E40" s="9" t="n">
-        <v>123</v>
+        <v>73</v>
       </c>
       <c r="F40" s="9" t="n">
         <v>183</v>
@@ -2496,17 +2636,21 @@
       </c>
       <c r="I40" s="21" t="n">
         <f aca="false">IF(SUM(B40:F40,H40)=0,"",SUM(B40:F40,H40))</f>
-        <v>1093</v>
+        <v>1043</v>
       </c>
       <c r="J40" s="21" t="n">
         <f aca="false">IF(I40="","",1440-I40)</f>
-        <v>347</v>
+        <v>397</v>
       </c>
       <c r="K40" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L40" s="22"/>
-      <c r="M40" s="22"/>
+      <c r="L40" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M40" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N40" s="23"/>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2523,7 +2667,7 @@
         <v>134</v>
       </c>
       <c r="E41" s="9" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>184</v>
@@ -2536,17 +2680,21 @@
       </c>
       <c r="I41" s="21" t="n">
         <f aca="false">IF(SUM(B41:F41,H41)=0,"",SUM(B41:F41,H41))</f>
-        <v>1099</v>
+        <v>1049</v>
       </c>
       <c r="J41" s="21" t="n">
         <f aca="false">IF(I41="","",1440-I41)</f>
-        <v>341</v>
+        <v>391</v>
       </c>
       <c r="K41" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
+      <c r="L41" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M41" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N41" s="23"/>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2563,7 +2711,7 @@
         <v>135</v>
       </c>
       <c r="E42" s="9" t="n">
-        <v>125</v>
+        <v>75</v>
       </c>
       <c r="F42" s="9" t="n">
         <v>185</v>
@@ -2576,17 +2724,21 @@
       </c>
       <c r="I42" s="21" t="n">
         <f aca="false">IF(SUM(B42:F42,H42)=0,"",SUM(B42:F42,H42))</f>
-        <v>1105</v>
+        <v>1055</v>
       </c>
       <c r="J42" s="21" t="n">
         <f aca="false">IF(I42="","",1440-I42)</f>
-        <v>335</v>
+        <v>385</v>
       </c>
       <c r="K42" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L42" s="22"/>
-      <c r="M42" s="22"/>
+      <c r="L42" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M42" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N42" s="23"/>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2603,7 +2755,7 @@
         <v>136</v>
       </c>
       <c r="E43" s="9" t="n">
-        <v>126</v>
+        <v>76</v>
       </c>
       <c r="F43" s="9" t="n">
         <v>186</v>
@@ -2616,17 +2768,21 @@
       </c>
       <c r="I43" s="21" t="n">
         <f aca="false">IF(SUM(B43:F43,H43)=0,"",SUM(B43:F43,H43))</f>
-        <v>1111</v>
+        <v>1061</v>
       </c>
       <c r="J43" s="21" t="n">
         <f aca="false">IF(I43="","",1440-I43)</f>
-        <v>329</v>
+        <v>379</v>
       </c>
       <c r="K43" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L43" s="22"/>
-      <c r="M43" s="22"/>
+      <c r="L43" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M43" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N43" s="23"/>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2665,8 +2821,12 @@
       <c r="K44" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L44" s="22"/>
-      <c r="M44" s="22"/>
+      <c r="L44" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M44" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N44" s="23"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2705,8 +2865,12 @@
       <c r="K45" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L45" s="22"/>
-      <c r="M45" s="22"/>
+      <c r="L45" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M45" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N45" s="23"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2745,8 +2909,12 @@
       <c r="K46" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L46" s="22"/>
-      <c r="M46" s="22"/>
+      <c r="L46" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M46" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N46" s="23"/>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2785,8 +2953,12 @@
       <c r="K47" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L47" s="22"/>
-      <c r="M47" s="22"/>
+      <c r="L47" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="M47" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N47" s="23"/>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2794,13 +2966,13 @@
         <v>46265</v>
       </c>
       <c r="B48" s="9" t="n">
-        <v>541</v>
+        <v>400</v>
       </c>
       <c r="C48" s="9" t="n">
         <v>71</v>
       </c>
       <c r="D48" s="9" t="n">
-        <v>141</v>
+        <v>80</v>
       </c>
       <c r="E48" s="9" t="n">
         <v>131</v>
@@ -2816,17 +2988,21 @@
       </c>
       <c r="I48" s="21" t="n">
         <f aca="false">IF(SUM(B48:F48,H48)=0,"",SUM(B48:F48,H48))</f>
-        <v>1141</v>
+        <v>939</v>
       </c>
       <c r="J48" s="21" t="n">
         <f aca="false">IF(I48="","",1440-I48)</f>
-        <v>299</v>
+        <v>501</v>
       </c>
       <c r="K48" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L48" s="22"/>
-      <c r="M48" s="22"/>
+      <c r="L48" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M48" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N48" s="23"/>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2834,19 +3010,19 @@
         <v>46266</v>
       </c>
       <c r="B49" s="9" t="n">
-        <v>542</v>
+        <v>401</v>
       </c>
       <c r="C49" s="9" t="n">
         <v>72</v>
       </c>
       <c r="D49" s="9" t="n">
-        <v>142</v>
+        <v>81</v>
       </c>
       <c r="E49" s="9" t="n">
         <v>132</v>
       </c>
       <c r="F49" s="9" t="n">
-        <v>192</v>
+        <v>140</v>
       </c>
       <c r="G49" s="9" t="n">
         <v>46</v>
@@ -2856,17 +3032,21 @@
       </c>
       <c r="I49" s="21" t="n">
         <f aca="false">IF(SUM(B49:F49,H49)=0,"",SUM(B49:F49,H49))</f>
-        <v>1147</v>
+        <v>893</v>
       </c>
       <c r="J49" s="21" t="n">
         <f aca="false">IF(I49="","",1440-I49)</f>
-        <v>293</v>
+        <v>547</v>
       </c>
       <c r="K49" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="L49" s="22"/>
-      <c r="M49" s="22"/>
+      <c r="L49" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="M49" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N49" s="23"/>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2874,39 +3054,43 @@
         <v>46267</v>
       </c>
       <c r="B50" s="9" t="n">
-        <v>543</v>
+        <v>402</v>
       </c>
       <c r="C50" s="9" t="n">
         <v>73</v>
       </c>
       <c r="D50" s="9" t="n">
-        <v>143</v>
+        <v>82</v>
       </c>
       <c r="E50" s="9" t="n">
         <v>133</v>
       </c>
       <c r="F50" s="9" t="n">
-        <v>193</v>
+        <v>141</v>
       </c>
       <c r="G50" s="9" t="n">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="H50" s="9" t="n">
         <v>68</v>
       </c>
       <c r="I50" s="21" t="n">
         <f aca="false">IF(SUM(B50:F50,H50)=0,"",SUM(B50:F50,H50))</f>
-        <v>1153</v>
+        <v>899</v>
       </c>
       <c r="J50" s="21" t="n">
         <f aca="false">IF(I50="","",1440-I50)</f>
-        <v>287</v>
+        <v>541</v>
       </c>
       <c r="K50" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L50" s="22"/>
-      <c r="M50" s="22"/>
+      <c r="L50" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M50" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N50" s="23"/>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2914,39 +3098,43 @@
         <v>46268</v>
       </c>
       <c r="B51" s="9" t="n">
-        <v>544</v>
+        <v>403</v>
       </c>
       <c r="C51" s="9" t="n">
         <v>74</v>
       </c>
       <c r="D51" s="9" t="n">
-        <v>144</v>
+        <v>83</v>
       </c>
       <c r="E51" s="9" t="n">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="F51" s="9" t="n">
-        <v>194</v>
+        <v>142</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="H51" s="9" t="n">
         <v>69</v>
       </c>
       <c r="I51" s="21" t="n">
         <f aca="false">IF(SUM(B51:F51,H51)=0,"",SUM(B51:F51,H51))</f>
-        <v>1159</v>
+        <v>891</v>
       </c>
       <c r="J51" s="21" t="n">
         <f aca="false">IF(I51="","",1440-I51)</f>
-        <v>281</v>
+        <v>549</v>
       </c>
       <c r="K51" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L51" s="22"/>
-      <c r="M51" s="22"/>
+      <c r="L51" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="M51" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N51" s="23"/>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2954,39 +3142,43 @@
         <v>46269</v>
       </c>
       <c r="B52" s="9" t="n">
-        <v>545</v>
+        <v>404</v>
       </c>
       <c r="C52" s="9" t="n">
         <v>75</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>145</v>
+        <v>84</v>
       </c>
       <c r="E52" s="9" t="n">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="F52" s="9" t="n">
-        <v>195</v>
+        <v>143</v>
       </c>
       <c r="G52" s="9" t="n">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="H52" s="9" t="n">
         <v>70</v>
       </c>
       <c r="I52" s="21" t="n">
         <f aca="false">IF(SUM(B52:F52,H52)=0,"",SUM(B52:F52,H52))</f>
-        <v>1165</v>
+        <v>897</v>
       </c>
       <c r="J52" s="21" t="n">
         <f aca="false">IF(I52="","",1440-I52)</f>
-        <v>275</v>
+        <v>543</v>
       </c>
       <c r="K52" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L52" s="22"/>
-      <c r="M52" s="22"/>
+      <c r="L52" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M52" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N52" s="23"/>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2994,7 +3186,7 @@
         <v>46270</v>
       </c>
       <c r="B53" s="9" t="n">
-        <v>546</v>
+        <v>405</v>
       </c>
       <c r="C53" s="9" t="n">
         <v>76</v>
@@ -3003,30 +3195,34 @@
         <v>146</v>
       </c>
       <c r="E53" s="9" t="n">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="F53" s="9" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="H53" s="9" t="n">
         <v>71</v>
       </c>
       <c r="I53" s="21" t="n">
         <f aca="false">IF(SUM(B53:F53,H53)=0,"",SUM(B53:F53,H53))</f>
-        <v>1171</v>
+        <v>964</v>
       </c>
       <c r="J53" s="21" t="n">
         <f aca="false">IF(I53="","",1440-I53)</f>
-        <v>269</v>
+        <v>476</v>
       </c>
       <c r="K53" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L53" s="22"/>
-      <c r="M53" s="22"/>
+      <c r="L53" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M53" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N53" s="23"/>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3043,30 +3239,34 @@
         <v>147</v>
       </c>
       <c r="E54" s="9" t="n">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>197</v>
+        <v>145</v>
       </c>
       <c r="G54" s="9" t="n">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="H54" s="9" t="n">
         <v>72</v>
       </c>
       <c r="I54" s="21" t="n">
         <f aca="false">IF(SUM(B54:F54,H54)=0,"",SUM(B54:F54,H54))</f>
-        <v>1177</v>
+        <v>1111</v>
       </c>
       <c r="J54" s="21" t="n">
         <f aca="false">IF(I54="","",1440-I54)</f>
-        <v>263</v>
+        <v>329</v>
       </c>
       <c r="K54" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L54" s="22"/>
-      <c r="M54" s="22"/>
+      <c r="L54" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M54" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N54" s="23"/>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3083,30 +3283,34 @@
         <v>148</v>
       </c>
       <c r="E55" s="9" t="n">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="F55" s="9" t="n">
-        <v>198</v>
+        <v>146</v>
       </c>
       <c r="G55" s="9" t="n">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="H55" s="9" t="n">
         <v>73</v>
       </c>
       <c r="I55" s="21" t="n">
         <f aca="false">IF(SUM(B55:F55,H55)=0,"",SUM(B55:F55,H55))</f>
-        <v>1183</v>
+        <v>1117</v>
       </c>
       <c r="J55" s="21" t="n">
         <f aca="false">IF(I55="","",1440-I55)</f>
-        <v>257</v>
+        <v>323</v>
       </c>
       <c r="K55" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L55" s="22"/>
-      <c r="M55" s="22"/>
+      <c r="L55" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M55" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N55" s="23"/>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3123,30 +3327,34 @@
         <v>149</v>
       </c>
       <c r="E56" s="9" t="n">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="F56" s="9" t="n">
-        <v>199</v>
+        <v>147</v>
       </c>
       <c r="G56" s="9" t="n">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="H56" s="9" t="n">
         <v>74</v>
       </c>
       <c r="I56" s="21" t="n">
         <f aca="false">IF(SUM(B56:F56,H56)=0,"",SUM(B56:F56,H56))</f>
-        <v>1189</v>
+        <v>1123</v>
       </c>
       <c r="J56" s="21" t="n">
         <f aca="false">IF(I56="","",1440-I56)</f>
-        <v>251</v>
+        <v>317</v>
       </c>
       <c r="K56" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L56" s="22"/>
-      <c r="M56" s="22"/>
+      <c r="L56" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M56" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N56" s="23"/>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3160,33 +3368,37 @@
         <v>80</v>
       </c>
       <c r="D57" s="9" t="n">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="E57" s="9" t="n">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="F57" s="9" t="n">
-        <v>200</v>
+        <v>148</v>
       </c>
       <c r="G57" s="9" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="H57" s="9" t="n">
         <v>75</v>
       </c>
       <c r="I57" s="21" t="n">
         <f aca="false">IF(SUM(B57:F57,H57)=0,"",SUM(B57:F57,H57))</f>
-        <v>1195</v>
+        <v>1049</v>
       </c>
       <c r="J57" s="21" t="n">
         <f aca="false">IF(I57="","",1440-I57)</f>
-        <v>245</v>
+        <v>391</v>
       </c>
       <c r="K57" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L57" s="22"/>
-      <c r="M57" s="22"/>
+      <c r="L57" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="M57" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N57" s="23"/>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3200,33 +3412,37 @@
         <v>81</v>
       </c>
       <c r="D58" s="9" t="n">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>201</v>
+        <v>149</v>
       </c>
       <c r="G58" s="9" t="n">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="H58" s="9" t="n">
         <v>76</v>
       </c>
       <c r="I58" s="21" t="n">
         <f aca="false">IF(SUM(B58:F58,H58)=0,"",SUM(B58:F58,H58))</f>
-        <v>1201</v>
+        <v>1055</v>
       </c>
       <c r="J58" s="21" t="n">
         <f aca="false">IF(I58="","",1440-I58)</f>
-        <v>239</v>
+        <v>385</v>
       </c>
       <c r="K58" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L58" s="22"/>
-      <c r="M58" s="22"/>
+      <c r="L58" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M58" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N58" s="23"/>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3240,33 +3456,37 @@
         <v>82</v>
       </c>
       <c r="D59" s="9" t="n">
-        <v>152</v>
+        <v>72</v>
       </c>
       <c r="E59" s="9" t="n">
         <v>142</v>
       </c>
       <c r="F59" s="9" t="n">
-        <v>202</v>
+        <v>150</v>
       </c>
       <c r="G59" s="9" t="n">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="H59" s="9" t="n">
         <v>77</v>
       </c>
       <c r="I59" s="21" t="n">
         <f aca="false">IF(SUM(B59:F59,H59)=0,"",SUM(B59:F59,H59))</f>
-        <v>1207</v>
+        <v>1075</v>
       </c>
       <c r="J59" s="21" t="n">
         <f aca="false">IF(I59="","",1440-I59)</f>
-        <v>233</v>
+        <v>365</v>
       </c>
       <c r="K59" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L59" s="22"/>
-      <c r="M59" s="22"/>
+      <c r="L59" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M59" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N59" s="23"/>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3280,33 +3500,37 @@
         <v>83</v>
       </c>
       <c r="D60" s="9" t="n">
-        <v>153</v>
+        <v>73</v>
       </c>
       <c r="E60" s="9" t="n">
         <v>143</v>
       </c>
       <c r="F60" s="9" t="n">
-        <v>203</v>
+        <v>151</v>
       </c>
       <c r="G60" s="9" t="n">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="H60" s="9" t="n">
         <v>78</v>
       </c>
       <c r="I60" s="21" t="n">
         <f aca="false">IF(SUM(B60:F60,H60)=0,"",SUM(B60:F60,H60))</f>
-        <v>1213</v>
+        <v>1081</v>
       </c>
       <c r="J60" s="21" t="n">
         <f aca="false">IF(I60="","",1440-I60)</f>
-        <v>227</v>
+        <v>359</v>
       </c>
       <c r="K60" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L60" s="22"/>
-      <c r="M60" s="22"/>
+      <c r="L60" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M60" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N60" s="23"/>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3320,13 +3544,13 @@
         <v>84</v>
       </c>
       <c r="D61" s="9" t="n">
-        <v>154</v>
+        <v>74</v>
       </c>
       <c r="E61" s="9" t="n">
         <v>144</v>
       </c>
       <c r="F61" s="9" t="n">
-        <v>204</v>
+        <v>120</v>
       </c>
       <c r="G61" s="9" t="n">
         <v>58</v>
@@ -3336,17 +3560,21 @@
       </c>
       <c r="I61" s="21" t="n">
         <f aca="false">IF(SUM(B61:F61,H61)=0,"",SUM(B61:F61,H61))</f>
-        <v>1219</v>
+        <v>1055</v>
       </c>
       <c r="J61" s="21" t="n">
         <f aca="false">IF(I61="","",1440-I61)</f>
-        <v>221</v>
+        <v>385</v>
       </c>
       <c r="K61" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L61" s="22"/>
-      <c r="M61" s="22"/>
+      <c r="L61" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M61" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N61" s="23"/>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3366,7 +3594,7 @@
         <v>145</v>
       </c>
       <c r="F62" s="9" t="n">
-        <v>205</v>
+        <v>121</v>
       </c>
       <c r="G62" s="9" t="n">
         <v>59</v>
@@ -3376,17 +3604,21 @@
       </c>
       <c r="I62" s="21" t="n">
         <f aca="false">IF(SUM(B62:F62,H62)=0,"",SUM(B62:F62,H62))</f>
-        <v>1225</v>
+        <v>1141</v>
       </c>
       <c r="J62" s="21" t="n">
         <f aca="false">IF(I62="","",1440-I62)</f>
-        <v>215</v>
+        <v>299</v>
       </c>
       <c r="K62" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L62" s="22"/>
-      <c r="M62" s="22"/>
+      <c r="L62" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M62" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N62" s="23"/>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3406,7 +3638,7 @@
         <v>146</v>
       </c>
       <c r="F63" s="9" t="n">
-        <v>206</v>
+        <v>122</v>
       </c>
       <c r="G63" s="9" t="n">
         <v>60</v>
@@ -3416,17 +3648,21 @@
       </c>
       <c r="I63" s="21" t="n">
         <f aca="false">IF(SUM(B63:F63,H63)=0,"",SUM(B63:F63,H63))</f>
-        <v>1231</v>
+        <v>1147</v>
       </c>
       <c r="J63" s="21" t="n">
         <f aca="false">IF(I63="","",1440-I63)</f>
-        <v>209</v>
+        <v>293</v>
       </c>
       <c r="K63" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L63" s="22"/>
-      <c r="M63" s="22"/>
+      <c r="L63" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="M63" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N63" s="23"/>
     </row>
     <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3446,7 +3682,7 @@
         <v>147</v>
       </c>
       <c r="F64" s="9" t="n">
-        <v>207</v>
+        <v>123</v>
       </c>
       <c r="G64" s="9" t="n">
         <v>61</v>
@@ -3456,17 +3692,21 @@
       </c>
       <c r="I64" s="21" t="n">
         <f aca="false">IF(SUM(B64:F64,H64)=0,"",SUM(B64:F64,H64))</f>
-        <v>1237</v>
+        <v>1153</v>
       </c>
       <c r="J64" s="21" t="n">
         <f aca="false">IF(I64="","",1440-I64)</f>
-        <v>203</v>
+        <v>287</v>
       </c>
       <c r="K64" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L64" s="22"/>
-      <c r="M64" s="22"/>
+      <c r="L64" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M64" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N64" s="23"/>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3486,7 +3726,7 @@
         <v>148</v>
       </c>
       <c r="F65" s="9" t="n">
-        <v>208</v>
+        <v>124</v>
       </c>
       <c r="G65" s="9" t="n">
         <v>62</v>
@@ -3496,17 +3736,21 @@
       </c>
       <c r="I65" s="21" t="n">
         <f aca="false">IF(SUM(B65:F65,H65)=0,"",SUM(B65:F65,H65))</f>
-        <v>1243</v>
+        <v>1159</v>
       </c>
       <c r="J65" s="21" t="n">
         <f aca="false">IF(I65="","",1440-I65)</f>
-        <v>197</v>
+        <v>281</v>
       </c>
       <c r="K65" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L65" s="22"/>
-      <c r="M65" s="22"/>
+      <c r="L65" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M65" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N65" s="23"/>
     </row>
     <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3526,7 +3770,7 @@
         <v>149</v>
       </c>
       <c r="F66" s="9" t="n">
-        <v>209</v>
+        <v>125</v>
       </c>
       <c r="G66" s="9" t="n">
         <v>63</v>
@@ -3536,17 +3780,21 @@
       </c>
       <c r="I66" s="21" t="n">
         <f aca="false">IF(SUM(B66:F66,H66)=0,"",SUM(B66:F66,H66))</f>
-        <v>1249</v>
+        <v>1165</v>
       </c>
       <c r="J66" s="21" t="n">
         <f aca="false">IF(I66="","",1440-I66)</f>
-        <v>191</v>
+        <v>275</v>
       </c>
       <c r="K66" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L66" s="22"/>
-      <c r="M66" s="22"/>
+      <c r="L66" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M66" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N66" s="23"/>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3566,7 +3814,7 @@
         <v>150</v>
       </c>
       <c r="F67" s="9" t="n">
-        <v>210</v>
+        <v>126</v>
       </c>
       <c r="G67" s="9" t="n">
         <v>64</v>
@@ -3576,17 +3824,21 @@
       </c>
       <c r="I67" s="21" t="n">
         <f aca="false">IF(SUM(B67:F67,H67)=0,"",SUM(B67:F67,H67))</f>
-        <v>1255</v>
+        <v>1171</v>
       </c>
       <c r="J67" s="21" t="n">
         <f aca="false">IF(I67="","",1440-I67)</f>
-        <v>185</v>
+        <v>269</v>
       </c>
       <c r="K67" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L67" s="22"/>
-      <c r="M67" s="22"/>
+      <c r="L67" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="M67" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N67" s="23"/>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3606,7 +3858,7 @@
         <v>151</v>
       </c>
       <c r="F68" s="9" t="n">
-        <v>211</v>
+        <v>127</v>
       </c>
       <c r="G68" s="9" t="n">
         <v>65</v>
@@ -3616,415 +3868,179 @@
       </c>
       <c r="I68" s="21" t="n">
         <f aca="false">IF(SUM(B68:F68,H68)=0,"",SUM(B68:F68,H68))</f>
-        <v>1261</v>
+        <v>1177</v>
       </c>
       <c r="J68" s="21" t="n">
         <f aca="false">IF(I68="","",1440-I68)</f>
-        <v>179</v>
+        <v>263</v>
       </c>
       <c r="K68" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="L68" s="22"/>
-      <c r="M68" s="22"/>
+      <c r="L68" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="M68" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="N68" s="23"/>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="20" t="n">
-        <v>46286</v>
-      </c>
-      <c r="B69" s="9" t="n">
-        <v>562</v>
-      </c>
-      <c r="C69" s="9" t="n">
-        <v>92</v>
-      </c>
-      <c r="D69" s="9" t="n">
-        <v>162</v>
-      </c>
-      <c r="E69" s="9" t="n">
-        <v>152</v>
-      </c>
-      <c r="F69" s="9" t="n">
-        <v>212</v>
-      </c>
-      <c r="G69" s="9" t="n">
-        <v>66</v>
-      </c>
-      <c r="H69" s="9" t="n">
-        <v>87</v>
-      </c>
-      <c r="I69" s="21" t="n">
-        <f aca="false">IF(SUM(B69:F69,H69)=0,"",SUM(B69:F69,H69))</f>
-        <v>1267</v>
-      </c>
-      <c r="J69" s="21" t="n">
-        <f aca="false">IF(I69="","",1440-I69)</f>
-        <v>173</v>
-      </c>
-      <c r="K69" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A69" s="20"/>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="9"/>
+      <c r="G69" s="9"/>
+      <c r="H69" s="9"/>
+      <c r="I69" s="21"/>
+      <c r="J69" s="21"/>
+      <c r="K69" s="22"/>
       <c r="L69" s="22"/>
       <c r="M69" s="22"/>
       <c r="N69" s="23"/>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="20" t="n">
-        <v>46287</v>
-      </c>
-      <c r="B70" s="9" t="n">
-        <v>563</v>
-      </c>
-      <c r="C70" s="9" t="n">
-        <v>93</v>
-      </c>
-      <c r="D70" s="9" t="n">
-        <v>163</v>
-      </c>
-      <c r="E70" s="9" t="n">
-        <v>153</v>
-      </c>
-      <c r="F70" s="9" t="n">
-        <v>213</v>
-      </c>
-      <c r="G70" s="9" t="n">
-        <v>67</v>
-      </c>
-      <c r="H70" s="9" t="n">
-        <v>88</v>
-      </c>
-      <c r="I70" s="21" t="n">
-        <f aca="false">IF(SUM(B70:F70,H70)=0,"",SUM(B70:F70,H70))</f>
-        <v>1273</v>
-      </c>
-      <c r="J70" s="21" t="n">
-        <f aca="false">IF(I70="","",1440-I70)</f>
-        <v>167</v>
-      </c>
-      <c r="K70" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A70" s="20"/>
+      <c r="B70" s="9"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="9"/>
+      <c r="F70" s="9"/>
+      <c r="G70" s="9"/>
+      <c r="H70" s="9"/>
+      <c r="I70" s="21"/>
+      <c r="J70" s="21"/>
+      <c r="K70" s="22"/>
       <c r="L70" s="22"/>
       <c r="M70" s="22"/>
       <c r="N70" s="23"/>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="20" t="n">
-        <v>46288</v>
-      </c>
-      <c r="B71" s="9" t="n">
-        <v>564</v>
-      </c>
-      <c r="C71" s="9" t="n">
-        <v>94</v>
-      </c>
-      <c r="D71" s="9" t="n">
-        <v>164</v>
-      </c>
-      <c r="E71" s="9" t="n">
-        <v>154</v>
-      </c>
-      <c r="F71" s="9" t="n">
-        <v>214</v>
-      </c>
-      <c r="G71" s="9" t="n">
-        <v>68</v>
-      </c>
-      <c r="H71" s="9" t="n">
-        <v>89</v>
-      </c>
-      <c r="I71" s="21" t="n">
-        <f aca="false">IF(SUM(B71:F71,H71)=0,"",SUM(B71:F71,H71))</f>
-        <v>1279</v>
-      </c>
-      <c r="J71" s="21" t="n">
-        <f aca="false">IF(I71="","",1440-I71)</f>
-        <v>161</v>
-      </c>
-      <c r="K71" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A71" s="20"/>
+      <c r="B71" s="9"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="9"/>
+      <c r="F71" s="9"/>
+      <c r="G71" s="9"/>
+      <c r="H71" s="9"/>
+      <c r="I71" s="21"/>
+      <c r="J71" s="21"/>
+      <c r="K71" s="22"/>
       <c r="L71" s="22"/>
       <c r="M71" s="22"/>
       <c r="N71" s="23"/>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="20" t="n">
-        <v>46289</v>
-      </c>
-      <c r="B72" s="9" t="n">
-        <v>565</v>
-      </c>
-      <c r="C72" s="9" t="n">
-        <v>95</v>
-      </c>
-      <c r="D72" s="9" t="n">
-        <v>165</v>
-      </c>
-      <c r="E72" s="9" t="n">
-        <v>155</v>
-      </c>
-      <c r="F72" s="9" t="n">
-        <v>215</v>
-      </c>
-      <c r="G72" s="9" t="n">
-        <v>69</v>
-      </c>
-      <c r="H72" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="I72" s="21" t="n">
-        <f aca="false">IF(SUM(B72:F72,H72)=0,"",SUM(B72:F72,H72))</f>
-        <v>1285</v>
-      </c>
-      <c r="J72" s="21" t="n">
-        <f aca="false">IF(I72="","",1440-I72)</f>
-        <v>155</v>
-      </c>
-      <c r="K72" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A72" s="20"/>
+      <c r="B72" s="9"/>
+      <c r="C72" s="9"/>
+      <c r="D72" s="9"/>
+      <c r="E72" s="9"/>
+      <c r="F72" s="9"/>
+      <c r="G72" s="9"/>
+      <c r="H72" s="9"/>
+      <c r="I72" s="21"/>
+      <c r="J72" s="21"/>
+      <c r="K72" s="22"/>
       <c r="L72" s="22"/>
       <c r="M72" s="22"/>
       <c r="N72" s="23"/>
     </row>
     <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="20" t="n">
-        <v>46290</v>
-      </c>
-      <c r="B73" s="9" t="n">
-        <v>566</v>
-      </c>
-      <c r="C73" s="9" t="n">
-        <v>96</v>
-      </c>
-      <c r="D73" s="9" t="n">
-        <v>166</v>
-      </c>
-      <c r="E73" s="9" t="n">
-        <v>156</v>
-      </c>
-      <c r="F73" s="9" t="n">
-        <v>216</v>
-      </c>
-      <c r="G73" s="9" t="n">
-        <v>70</v>
-      </c>
-      <c r="H73" s="9" t="n">
-        <v>91</v>
-      </c>
-      <c r="I73" s="21" t="n">
-        <f aca="false">IF(SUM(B73:F73,H73)=0,"",SUM(B73:F73,H73))</f>
-        <v>1291</v>
-      </c>
-      <c r="J73" s="21" t="n">
-        <f aca="false">IF(I73="","",1440-I73)</f>
-        <v>149</v>
-      </c>
-      <c r="K73" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A73" s="20"/>
+      <c r="B73" s="9"/>
+      <c r="C73" s="9"/>
+      <c r="D73" s="9"/>
+      <c r="E73" s="9"/>
+      <c r="F73" s="9"/>
+      <c r="G73" s="9"/>
+      <c r="H73" s="9"/>
+      <c r="I73" s="21"/>
+      <c r="J73" s="21"/>
+      <c r="K73" s="22"/>
       <c r="L73" s="22"/>
       <c r="M73" s="22"/>
       <c r="N73" s="23"/>
     </row>
     <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="20" t="n">
-        <v>46291</v>
-      </c>
-      <c r="B74" s="9" t="n">
-        <v>567</v>
-      </c>
-      <c r="C74" s="9" t="n">
-        <v>97</v>
-      </c>
-      <c r="D74" s="9" t="n">
-        <v>167</v>
-      </c>
-      <c r="E74" s="9" t="n">
-        <v>157</v>
-      </c>
-      <c r="F74" s="9" t="n">
-        <v>217</v>
-      </c>
-      <c r="G74" s="9" t="n">
-        <v>71</v>
-      </c>
-      <c r="H74" s="9" t="n">
-        <v>92</v>
-      </c>
-      <c r="I74" s="21" t="n">
-        <f aca="false">IF(SUM(B74:F74,H74)=0,"",SUM(B74:F74,H74))</f>
-        <v>1297</v>
-      </c>
-      <c r="J74" s="21" t="n">
-        <f aca="false">IF(I74="","",1440-I74)</f>
-        <v>143</v>
-      </c>
-      <c r="K74" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A74" s="20"/>
+      <c r="B74" s="9"/>
+      <c r="C74" s="9"/>
+      <c r="D74" s="9"/>
+      <c r="E74" s="9"/>
+      <c r="F74" s="9"/>
+      <c r="G74" s="9"/>
+      <c r="H74" s="9"/>
+      <c r="I74" s="21"/>
+      <c r="J74" s="21"/>
+      <c r="K74" s="22"/>
       <c r="L74" s="22"/>
       <c r="M74" s="22"/>
       <c r="N74" s="23"/>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="20" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B75" s="9" t="n">
-        <v>568</v>
-      </c>
-      <c r="C75" s="9" t="n">
-        <v>98</v>
-      </c>
-      <c r="D75" s="9" t="n">
-        <v>168</v>
-      </c>
-      <c r="E75" s="9" t="n">
-        <v>158</v>
-      </c>
-      <c r="F75" s="9" t="n">
-        <v>218</v>
-      </c>
-      <c r="G75" s="9" t="n">
-        <v>72</v>
-      </c>
-      <c r="H75" s="9" t="n">
-        <v>93</v>
-      </c>
-      <c r="I75" s="21" t="n">
-        <f aca="false">IF(SUM(B75:F75,H75)=0,"",SUM(B75:F75,H75))</f>
-        <v>1303</v>
-      </c>
-      <c r="J75" s="21" t="n">
-        <f aca="false">IF(I75="","",1440-I75)</f>
-        <v>137</v>
-      </c>
-      <c r="K75" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A75" s="20"/>
+      <c r="B75" s="9"/>
+      <c r="C75" s="9"/>
+      <c r="D75" s="9"/>
+      <c r="E75" s="9"/>
+      <c r="F75" s="9"/>
+      <c r="G75" s="9"/>
+      <c r="H75" s="9"/>
+      <c r="I75" s="21"/>
+      <c r="J75" s="21"/>
+      <c r="K75" s="22"/>
       <c r="L75" s="22"/>
       <c r="M75" s="22"/>
       <c r="N75" s="23"/>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="20" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B76" s="9" t="n">
-        <v>569</v>
-      </c>
-      <c r="C76" s="9" t="n">
-        <v>99</v>
-      </c>
-      <c r="D76" s="9" t="n">
-        <v>169</v>
-      </c>
-      <c r="E76" s="9" t="n">
-        <v>159</v>
-      </c>
-      <c r="F76" s="9" t="n">
-        <v>219</v>
-      </c>
-      <c r="G76" s="9" t="n">
-        <v>73</v>
-      </c>
-      <c r="H76" s="9" t="n">
-        <v>94</v>
-      </c>
-      <c r="I76" s="21" t="n">
-        <f aca="false">IF(SUM(B76:F76,H76)=0,"",SUM(B76:F76,H76))</f>
-        <v>1309</v>
-      </c>
-      <c r="J76" s="21" t="n">
-        <f aca="false">IF(I76="","",1440-I76)</f>
-        <v>131</v>
-      </c>
-      <c r="K76" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A76" s="20"/>
+      <c r="B76" s="9"/>
+      <c r="C76" s="9"/>
+      <c r="D76" s="9"/>
+      <c r="E76" s="9"/>
+      <c r="F76" s="9"/>
+      <c r="G76" s="9"/>
+      <c r="H76" s="9"/>
+      <c r="I76" s="21"/>
+      <c r="J76" s="21"/>
+      <c r="K76" s="22"/>
       <c r="L76" s="22"/>
       <c r="M76" s="22"/>
       <c r="N76" s="23"/>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="20" t="n">
-        <v>46294</v>
-      </c>
-      <c r="B77" s="9" t="n">
-        <v>570</v>
-      </c>
-      <c r="C77" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="D77" s="9" t="n">
-        <v>170</v>
-      </c>
-      <c r="E77" s="9" t="n">
-        <v>160</v>
-      </c>
-      <c r="F77" s="9" t="n">
-        <v>220</v>
-      </c>
-      <c r="G77" s="9" t="n">
-        <v>74</v>
-      </c>
-      <c r="H77" s="9" t="n">
-        <v>95</v>
-      </c>
-      <c r="I77" s="21" t="n">
-        <f aca="false">IF(SUM(B77:F77,H77)=0,"",SUM(B77:F77,H77))</f>
-        <v>1315</v>
-      </c>
-      <c r="J77" s="21" t="n">
-        <f aca="false">IF(I77="","",1440-I77)</f>
-        <v>125</v>
-      </c>
-      <c r="K77" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A77" s="20"/>
+      <c r="B77" s="9"/>
+      <c r="C77" s="9"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="9"/>
+      <c r="F77" s="9"/>
+      <c r="G77" s="9"/>
+      <c r="H77" s="9"/>
+      <c r="I77" s="21"/>
+      <c r="J77" s="21"/>
+      <c r="K77" s="22"/>
       <c r="L77" s="22"/>
       <c r="M77" s="22"/>
       <c r="N77" s="23"/>
     </row>
     <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="20" t="n">
-        <v>46295</v>
-      </c>
-      <c r="B78" s="9" t="n">
-        <v>571</v>
-      </c>
-      <c r="C78" s="9" t="n">
-        <v>101</v>
-      </c>
-      <c r="D78" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="E78" s="9" t="n">
-        <v>161</v>
-      </c>
-      <c r="F78" s="9" t="n">
-        <v>221</v>
-      </c>
-      <c r="G78" s="9" t="n">
-        <v>75</v>
-      </c>
-      <c r="H78" s="9" t="n">
-        <v>96</v>
-      </c>
-      <c r="I78" s="21" t="n">
-        <f aca="false">IF(SUM(B78:F78,H78)=0,"",SUM(B78:F78,H78))</f>
-        <v>1321</v>
-      </c>
-      <c r="J78" s="21" t="n">
-        <f aca="false">IF(I78="","",1440-I78)</f>
-        <v>119</v>
-      </c>
-      <c r="K78" s="22" t="s">
-        <v>56</v>
-      </c>
+      <c r="A78" s="20"/>
+      <c r="B78" s="9"/>
+      <c r="C78" s="9"/>
+      <c r="D78" s="9"/>
+      <c r="E78" s="9"/>
+      <c r="F78" s="9"/>
+      <c r="G78" s="9"/>
+      <c r="H78" s="9"/>
+      <c r="I78" s="21"/>
+      <c r="J78" s="21"/>
+      <c r="K78" s="22"/>
       <c r="L78" s="22"/>
       <c r="M78" s="22"/>
       <c r="N78" s="23"/>
@@ -4038,14 +4054,8 @@
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
       <c r="H79" s="9"/>
-      <c r="I79" s="21" t="str">
-        <f aca="false">IF(SUM(B79:F79,H79)=0,"",SUM(B79:F79,H79))</f>
-        <v/>
-      </c>
-      <c r="J79" s="21" t="str">
-        <f aca="false">IF(I79="","",1440-I79)</f>
-        <v/>
-      </c>
+      <c r="I79" s="21"/>
+      <c r="J79" s="21"/>
       <c r="K79" s="22"/>
       <c r="L79" s="22"/>
       <c r="M79" s="22"/>

</xml_diff>